<commit_message>
auto update 21/04/2026  6.00.23,10
</commit_message>
<xml_diff>
--- a/output/Rekap RUP Tahun 2026 (2026-04-21) Legacy.xlsx
+++ b/output/Rekap RUP Tahun 2026 (2026-04-21) Legacy.xlsx
@@ -461,7 +461,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Badan Kepegawaian dan Pengembangan Sumber Daya Manusiaâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Badan Kepegawaian dan Pengembangan Sumber Daya Manusiaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -489,7 +489,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Badan Kesatuan Bangsa dan Politikâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Badan Kesatuan Bangsa dan Politikâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -517,7 +517,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Badan Keuangan dan Aset Daerahâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Badan Keuangan dan Aset Daerahâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -545,7 +545,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Badan Penanggulangan Bencana Daerahâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Badan Penanggulangan Bencana Daerahâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -573,7 +573,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Badan Pendapatan Daerahâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Badan Pendapatan Daerahâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -601,7 +601,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Badan Perencanaan Pembangunan, Riset dan Inovasi Daerahâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Badan Perencanaan Pembangunan, Riset dan Inovasi Daerahâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -629,7 +629,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Balai Latihan Kerjaâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Balai Latihan Kerjaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -657,7 +657,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Dermaga Indera Sariâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Dermaga Indera Sariâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -685,7 +685,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Dinas Kepemudaan dan Olahragaâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Dinas Kepemudaan dan Olahragaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -713,7 +713,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Dinas Kependudukan dan Pencatatan Sipilâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Dinas Kependudukan dan Pencatatan Sipilâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -741,7 +741,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Dinas Kesehatanâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Dinas Kesehatanâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -769,7 +769,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Dinas Komunikasi, Informatika, Statistik dan Persandianâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Dinas Komunikasi, Informatika, Statistik dan Persandianâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -797,7 +797,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Dinas Lingkungan Hidupâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Dinas Lingkungan Hidupâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -825,7 +825,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Dinas Pariwisataâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Dinas Pariwisataâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -853,7 +853,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Dinas Pekerjaan Umum dan Penataan Ruangâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Dinas Pekerjaan Umum dan Penataan Ruangâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -881,7 +881,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Dinas Pemadam Kebakaran dan Penyelamatanâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Dinas Pemadam Kebakaran dan Penyelamatanâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -909,7 +909,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Dinas Pemberdayaan Masyarakat dan Desaâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Dinas Pemberdayaan Masyarakat dan Desaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -937,7 +937,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Dinas Pemberdayaan Perempuan dan Perlindungan Anak, Pengendalian Penduduk dan Keluarga Berencanaâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Dinas Pemberdayaan Perempuan dan Perlindungan Anak, Pengendalian Penduduk dan Keluarga Berencanaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -965,7 +965,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Dinas Penanaman Modal dan Pelayanan Terpadu Satu Pintuâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Dinas Penanaman Modal dan Pelayanan Terpadu Satu Pintuâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -993,7 +993,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Dinas Pendidikan dan Kebudayaanâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Dinas Pendidikan dan Kebudayaanâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1021,7 +1021,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Dinas Perhubunganâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Dinas Perhubunganâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1049,7 +1049,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Dinas Perikanan dan Ketahanan Panganâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Dinas Perikanan dan Ketahanan Panganâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1077,7 +1077,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Dinas Perindustrian, Perdagangan, Koperasi, Usaha Kecil dan Menengahâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Dinas Perindustrian, Perdagangan, Koperasi, Usaha Kecil dan Menengahâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1105,7 +1105,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Dinas Perpustakaan dan Kearsipanâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Dinas Perpustakaan dan Kearsipanâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1133,7 +1133,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Dinas Pertanianâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Dinas Pertanianâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1161,7 +1161,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Dinas Perumahan Rakyat, Kawasan Pemukiman dan Pertanahanâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Dinas Perumahan Rakyat, Kawasan Pemukiman dan Pertanahanâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1189,7 +1189,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Dinas Sosialâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Dinas Sosialâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1217,7 +1217,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Dinas Tenaga Kerja dan Transmigrasiâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Dinas Tenaga Kerja dan Transmigrasiâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1245,7 +1245,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Inspektorat Daerahâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Inspektorat Daerahâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1273,7 +1273,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Instalasi Farmasiâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Instalasi Farmasiâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1301,7 +1301,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Kecamatan Arut Selatanâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Kecamatan Arut Selatanâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1329,7 +1329,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Kecamatan Arut Utaraâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Kecamatan Arut Utaraâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1357,7 +1357,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Kecamatan Kotawaringin Lamaâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Kecamatan Kotawaringin Lamaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1385,7 +1385,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Kecamatan Kumaiâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Kecamatan Kumaiâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1413,7 +1413,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Kecamatan Pangkalan Bantengâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Kecamatan Pangkalan Bantengâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1441,7 +1441,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Kecamatan Pangkalan Ladaâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Kecamatan Pangkalan Ladaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1469,7 +1469,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Kelurahan Baruâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Kelurahan Baruâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1497,7 +1497,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Kelurahan Candiâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Kelurahan Candiâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1525,7 +1525,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Kelurahan Kotawaringin Hilirâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Kelurahan Kotawaringin Hilirâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1553,7 +1553,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Kelurahan Kotawaringin Huluâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Kelurahan Kotawaringin Huluâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1581,7 +1581,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Kelurahan Kumai Hilirâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Kelurahan Kumai Hilirâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1609,7 +1609,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Kelurahan Kumai Huluâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Kelurahan Kumai Huluâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1637,7 +1637,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Kelurahan Madurejoâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Kelurahan Madurejoâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1665,7 +1665,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Kelurahan Mendawai Seberangâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Kelurahan Mendawai Seberangâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1693,7 +1693,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Kelurahan Mendawaiâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Kelurahan Mendawaiâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1721,7 +1721,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Kelurahan Pangkutâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Kelurahan Pangkutâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1749,7 +1749,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Kelurahan Raja Seberangâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Kelurahan Raja Seberangâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1777,7 +1777,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Kelurahan Rajaâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Kelurahan Rajaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1805,7 +1805,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Kelurahan Sidorejoâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Kelurahan Sidorejoâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1833,7 +1833,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Laboratorium Bahan Konstruksiâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Laboratorium Bahan Konstruksiâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1861,7 +1861,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Laboratorium Kesehatan Daerahâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Laboratorium Kesehatan Daerahâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1889,7 +1889,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Laboratorium Lingkunganâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Laboratorium Lingkunganâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1917,7 +1917,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Pelabuhan Penyeberangan Kumaiâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Pelabuhan Penyeberangan Kumaiâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1945,7 +1945,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Pengembangan Pakan dan Ternak Unggulâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Pengembangan Pakan dan Ternak Unggulâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1973,7 +1973,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Pengujian Kendaraan Bermotorâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Pengujian Kendaraan Bermotorâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -2001,7 +2001,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Puskesmas Arut Selatanâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Puskesmas Arut Selatanâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2029,7 +2029,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Puskesmas Arut Utaraâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Puskesmas Arut Utaraâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -2057,7 +2057,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Puskesmas Ipuh Bangun Jayaâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Puskesmas Ipuh Bangun Jayaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -2085,7 +2085,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Puskesmas Karang Mulyaâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Puskesmas Karang Mulyaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -2113,7 +2113,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Puskesmas Kotawaringin Lamaâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Puskesmas Kotawaringin Lamaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -2141,7 +2141,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Puskesmas Kumaiâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Puskesmas Kumaiâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -2169,7 +2169,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Puskesmas Kumpai Batu Atasâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Puskesmas Kumpai Batu Atasâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -2197,7 +2197,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Puskesmas Madurejoâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Puskesmas Madurejoâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -2225,7 +2225,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Puskesmas Mendawaiâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Puskesmas Mendawaiâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -2253,7 +2253,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Puskesmas Natai Pelingkauâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Puskesmas Natai Pelingkauâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -2281,7 +2281,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Puskesmas Pandu Sanjayaâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Puskesmas Pandu Sanjayaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -2309,7 +2309,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Puskesmas Pangkalan Ladaâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Puskesmas Pangkalan Ladaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -2337,7 +2337,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Puskesmas Riam Durianâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Puskesmas Riam Durianâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -2365,7 +2365,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Puskesmas Runtuâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Puskesmas Runtuâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -2393,7 +2393,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Puskesmas Sambiâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Puskesmas Sambiâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -2421,7 +2421,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Puskesmas Semanggangâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Puskesmas Semanggangâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -2449,7 +2449,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Puskesmas Sungai Rangitâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Puskesmas Sungai Rangitâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -2477,7 +2477,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Puskesmas Teluk Bogamâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Puskesmas Teluk Bogamâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -2505,7 +2505,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Rumah Potong Hewan Ruminansiaâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Rumah Potong Hewan Ruminansiaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -2533,7 +2533,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Rumah Sakit Kutaringinâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Rumah Sakit Kutaringinâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -2561,7 +2561,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Rumah Sakit Umum Daerah Sultan Imanuddinâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Rumah Sakit Umum Daerah Sultan Imanuddinâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -2589,7 +2589,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Satuan Polisi Pamong Prajaâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Satuan Polisi Pamong Prajaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -2617,7 +2617,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Sekretariat Daerahâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Sekretariat Daerahâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -2645,7 +2645,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Sekretariat DPRDâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Sekretariat DPRDâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -2673,7 +2673,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Workshop dan Peralatan Konstruksiâ£âââââ âââââââââ ââââ ââââ ââââââââââââ âââââ â âââââââââââ ââââââ ââââââââ â âââ¤</t>
+          <t>Workshop dan Peralatan Konstruksiâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
         </is>
       </c>
       <c r="B81" t="n">

</xml_diff>

<commit_message>
auto update 21/04/2026  7.00.27,70
</commit_message>
<xml_diff>
--- a/output/Rekap RUP Tahun 2026 (2026-04-21) Legacy.xlsx
+++ b/output/Rekap RUP Tahun 2026 (2026-04-21) Legacy.xlsx
@@ -461,7 +461,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Badan Kepegawaian dan Pengembangan Sumber Daya Manusiaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Badan Kepegawaian dan Pengembangan Sumber Daya Manusia</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -489,7 +489,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Badan Kesatuan Bangsa dan Politikâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Badan Kesatuan Bangsa dan Politik</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -517,7 +517,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Badan Keuangan dan Aset Daerahâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Badan Keuangan dan Aset Daerah</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -545,7 +545,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Badan Penanggulangan Bencana Daerahâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Badan Penanggulangan Bencana Daerah</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -573,7 +573,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Badan Pendapatan Daerahâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Badan Pendapatan Daerah</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -601,7 +601,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Badan Perencanaan Pembangunan, Riset dan Inovasi Daerahâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Badan Perencanaan Pembangunan, Riset dan Inovasi Daerah</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -629,7 +629,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Balai Latihan Kerjaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Balai Latihan Kerja</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -657,7 +657,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Dermaga Indera Sariâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Dermaga Indera Sari</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -685,7 +685,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Dinas Kepemudaan dan Olahragaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Dinas Kepemudaan dan Olahraga</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -713,7 +713,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Dinas Kependudukan dan Pencatatan Sipilâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Dinas Kependudukan dan Pencatatan Sipil</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -741,7 +741,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Dinas Kesehatanâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Dinas Kesehatan</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -769,7 +769,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Dinas Komunikasi, Informatika, Statistik dan Persandianâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Dinas Komunikasi, Informatika, Statistik dan Persandian</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -797,7 +797,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Dinas Lingkungan Hidupâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Dinas Lingkungan Hidup</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -825,7 +825,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Dinas Pariwisataâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Dinas Pariwisata</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -853,7 +853,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Dinas Pekerjaan Umum dan Penataan Ruangâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Dinas Pekerjaan Umum dan Penataan Ruang</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -881,7 +881,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Dinas Pemadam Kebakaran dan Penyelamatanâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Dinas Pemadam Kebakaran dan Penyelamatan</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -909,7 +909,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Dinas Pemberdayaan Masyarakat dan Desaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Dinas Pemberdayaan Masyarakat dan Desa</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -937,7 +937,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Dinas Pemberdayaan Perempuan dan Perlindungan Anak, Pengendalian Penduduk dan Keluarga Berencanaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Dinas Pemberdayaan Perempuan dan Perlindungan Anak, Pengendalian Penduduk dan Keluarga Berencana</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -965,7 +965,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Dinas Penanaman Modal dan Pelayanan Terpadu Satu Pintuâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Dinas Penanaman Modal dan Pelayanan Terpadu Satu Pintu</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -993,7 +993,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Dinas Pendidikan dan Kebudayaanâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Dinas Pendidikan dan Kebudayaan</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1021,7 +1021,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Dinas Perhubunganâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Dinas Perhubungan</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1049,7 +1049,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Dinas Perikanan dan Ketahanan Panganâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Dinas Perikanan dan Ketahanan Pangan</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1077,7 +1077,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Dinas Perindustrian, Perdagangan, Koperasi, Usaha Kecil dan Menengahâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Dinas Perindustrian, Perdagangan, Koperasi, Usaha Kecil dan Menengah</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1105,7 +1105,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Dinas Perpustakaan dan Kearsipanâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Dinas Perpustakaan dan Kearsipan</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1133,7 +1133,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Dinas Pertanianâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Dinas Pertanian</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1161,7 +1161,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Dinas Perumahan Rakyat, Kawasan Pemukiman dan Pertanahanâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Dinas Perumahan Rakyat, Kawasan Pemukiman dan Pertanahan</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1189,7 +1189,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Dinas Sosialâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Dinas Sosial</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1217,7 +1217,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Dinas Tenaga Kerja dan Transmigrasiâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Dinas Tenaga Kerja dan Transmigrasi</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1245,7 +1245,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Inspektorat Daerahâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Inspektorat Daerah</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1273,7 +1273,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Instalasi Farmasiâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Instalasi Farmasi</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1301,7 +1301,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Kecamatan Arut Selatanâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Kecamatan Arut Selatan</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1329,7 +1329,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Kecamatan Arut Utaraâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Kecamatan Arut Utara</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1357,7 +1357,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Kecamatan Kotawaringin Lamaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Kecamatan Kotawaringin Lama</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1385,7 +1385,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Kecamatan Kumaiâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Kecamatan Kumai</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1413,7 +1413,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Kecamatan Pangkalan Bantengâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Kecamatan Pangkalan Banteng</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1441,7 +1441,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Kecamatan Pangkalan Ladaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Kecamatan Pangkalan Lada</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1469,7 +1469,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Kelurahan Baruâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Kelurahan Baru</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1497,7 +1497,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Kelurahan Candiâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Kelurahan Candi</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1525,7 +1525,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Kelurahan Kotawaringin Hilirâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Kelurahan Kotawaringin Hilir</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1553,7 +1553,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Kelurahan Kotawaringin Huluâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Kelurahan Kotawaringin Hulu</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1581,7 +1581,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Kelurahan Kumai Hilirâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Kelurahan Kumai Hilir</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1609,7 +1609,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Kelurahan Kumai Huluâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Kelurahan Kumai Hulu</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1637,7 +1637,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Kelurahan Madurejoâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Kelurahan Madurejo</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1665,7 +1665,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Kelurahan Mendawai Seberangâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Kelurahan Mendawai</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1693,7 +1693,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Kelurahan Mendawaiâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Kelurahan Mendawai Seberang</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1721,7 +1721,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Kelurahan Pangkutâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Kelurahan Pangkut</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1749,7 +1749,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Kelurahan Raja Seberangâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Kelurahan Raja</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1777,7 +1777,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Kelurahan Rajaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Kelurahan Raja Seberang</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1805,7 +1805,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Kelurahan Sidorejoâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Kelurahan Sidorejo</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1833,7 +1833,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Laboratorium Bahan Konstruksiâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Laboratorium Bahan Konstruksi</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1861,7 +1861,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Laboratorium Kesehatan Daerahâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Laboratorium Kesehatan Daerah</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1889,7 +1889,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Laboratorium Lingkunganâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Laboratorium Lingkungan</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1917,7 +1917,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Pelabuhan Penyeberangan Kumaiâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Pelabuhan Penyeberangan Kumai</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1945,7 +1945,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Pengembangan Pakan dan Ternak Unggulâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Pengembangan Pakan dan Ternak Unggul</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1973,7 +1973,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Pengujian Kendaraan Bermotorâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Pengujian Kendaraan Bermotor</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -2001,7 +2001,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Puskesmas Arut Selatanâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Puskesmas Arut Selatan</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2029,7 +2029,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Puskesmas Arut Utaraâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Puskesmas Arut Utara</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -2057,7 +2057,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Puskesmas Ipuh Bangun Jayaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Puskesmas Ipuh Bangun Jaya</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -2085,7 +2085,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Puskesmas Karang Mulyaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Puskesmas Karang Mulya</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -2113,7 +2113,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Puskesmas Kotawaringin Lamaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Puskesmas Kotawaringin Lama</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -2141,7 +2141,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Puskesmas Kumaiâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Puskesmas Kumai</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -2169,7 +2169,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Puskesmas Kumpai Batu Atasâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Puskesmas Kumpai Batu Atas</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -2197,7 +2197,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Puskesmas Madurejoâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Puskesmas Madurejo</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -2225,7 +2225,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Puskesmas Mendawaiâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Puskesmas Mendawai</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -2253,7 +2253,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Puskesmas Natai Pelingkauâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Puskesmas Natai Pelingkau</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -2281,7 +2281,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Puskesmas Pandu Sanjayaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Puskesmas Pandu Sanjaya</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -2309,7 +2309,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Puskesmas Pangkalan Ladaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Puskesmas Pangkalan Lada</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -2337,7 +2337,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Puskesmas Riam Durianâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Puskesmas Riam Durian</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -2365,7 +2365,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Puskesmas Runtuâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Puskesmas Runtu</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -2393,7 +2393,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Puskesmas Sambiâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Puskesmas Sambi</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -2421,7 +2421,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Puskesmas Semanggangâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Puskesmas Semanggang</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -2449,7 +2449,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Puskesmas Sungai Rangitâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Puskesmas Sungai Rangit</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -2477,7 +2477,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Puskesmas Teluk Bogamâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Puskesmas Teluk Bogam</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -2505,7 +2505,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Rumah Potong Hewan Ruminansiaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Rumah Potong Hewan Ruminansia</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -2533,7 +2533,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Rumah Sakit Kutaringinâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Rumah Sakit Kutaringin</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -2561,7 +2561,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Rumah Sakit Umum Daerah Sultan Imanuddinâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Rumah Sakit Umum Daerah Sultan Imanuddin</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -2589,7 +2589,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Satuan Polisi Pamong Prajaâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Satuan Polisi Pamong Praja</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -2617,7 +2617,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Sekretariat Daerahâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Sekretariat Daerah</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -2645,7 +2645,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Sekretariat DPRDâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Sekretariat DPRD</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -2673,7 +2673,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Workshop dan Peralatan Konstruksiâ£ââââââ â ââ âââââ ââââââââ ââ ââââ ââââ â ââââââ ââââââââââââ ââ âââââ ââââââ ââ ââ â¤</t>
+          <t>Workshop dan Peralatan Konstruksi</t>
         </is>
       </c>
       <c r="B81" t="n">

</xml_diff>

<commit_message>
auto update 21/04/2026  9.00.24,96
</commit_message>
<xml_diff>
--- a/output/Rekap RUP Tahun 2026 (2026-04-21) Legacy.xlsx
+++ b/output/Rekap RUP Tahun 2026 (2026-04-21) Legacy.xlsx
@@ -461,7 +461,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Badan Kepegawaian dan Pengembangan Sumber Daya Manusia</t>
+          <t>Badan Kepegawaian dan Pengembangan Sumber Daya Manusiaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -489,7 +489,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Badan Kesatuan Bangsa dan Politik</t>
+          <t>Badan Kesatuan Bangsa dan Politikâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -517,7 +517,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Badan Keuangan dan Aset Daerah</t>
+          <t>Badan Keuangan dan Aset Daerahâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -545,7 +545,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Badan Penanggulangan Bencana Daerah</t>
+          <t>Badan Penanggulangan Bencana Daerahâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -573,7 +573,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Badan Pendapatan Daerah</t>
+          <t>Badan Pendapatan Daerahâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -601,7 +601,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Badan Perencanaan Pembangunan, Riset dan Inovasi Daerah</t>
+          <t>Badan Perencanaan Pembangunan, Riset dan Inovasi Daerahâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -629,7 +629,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Balai Latihan Kerja</t>
+          <t>Balai Latihan Kerjaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -657,7 +657,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Dermaga Indera Sari</t>
+          <t>Dermaga Indera Sariâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -685,7 +685,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Dinas Kepemudaan dan Olahraga</t>
+          <t>Dinas Kepemudaan dan Olahragaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -713,7 +713,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Dinas Kependudukan dan Pencatatan Sipil</t>
+          <t>Dinas Kependudukan dan Pencatatan Sipilâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -741,7 +741,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Dinas Kesehatan</t>
+          <t>Dinas Kesehatanâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -769,11 +769,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Dinas Komunikasi, Informatika, Statistik dan Persandian</t>
+          <t>Dinas Komunikasi, Informatika, Statistik dan Persandianâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>7585371581</v>
+        <v>4809371581</v>
       </c>
       <c r="C13" t="n">
         <v>4363300381</v>
@@ -797,7 +797,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Dinas Lingkungan Hidup</t>
+          <t>Dinas Lingkungan Hidupâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -825,7 +825,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Dinas Pariwisata</t>
+          <t>Dinas Pariwisataâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -853,11 +853,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Dinas Pekerjaan Umum dan Penataan Ruang</t>
+          <t>Dinas Pekerjaan Umum dan Penataan Ruangâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>106337273694</v>
+        <v>105714344580</v>
       </c>
       <c r="C16" t="n">
         <v>105032048100</v>
@@ -881,7 +881,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Dinas Pemadam Kebakaran dan Penyelamatan</t>
+          <t>Dinas Pemadam Kebakaran dan Penyelamatanâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -909,7 +909,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Dinas Pemberdayaan Masyarakat dan Desa</t>
+          <t>Dinas Pemberdayaan Masyarakat dan Desaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -937,7 +937,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Dinas Pemberdayaan Perempuan dan Perlindungan Anak, Pengendalian Penduduk dan Keluarga Berencana</t>
+          <t>Dinas Pemberdayaan Perempuan dan Perlindungan Anak, Pengendalian Penduduk dan Keluarga Berencanaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -965,7 +965,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Dinas Penanaman Modal dan Pelayanan Terpadu Satu Pintu</t>
+          <t>Dinas Penanaman Modal dan Pelayanan Terpadu Satu Pintuâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -993,7 +993,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Dinas Pendidikan dan Kebudayaan</t>
+          <t>Dinas Pendidikan dan Kebudayaanâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1021,7 +1021,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Dinas Perhubungan</t>
+          <t>Dinas Perhubunganâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1049,7 +1049,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Dinas Perikanan dan Ketahanan Pangan</t>
+          <t>Dinas Perikanan dan Ketahanan Panganâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1077,7 +1077,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Dinas Perindustrian, Perdagangan, Koperasi, Usaha Kecil dan Menengah</t>
+          <t>Dinas Perindustrian, Perdagangan, Koperasi, Usaha Kecil dan Menengahâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1105,7 +1105,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Dinas Perpustakaan dan Kearsipan</t>
+          <t>Dinas Perpustakaan dan Kearsipanâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1133,7 +1133,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Dinas Pertanian</t>
+          <t>Dinas Pertanianâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1161,7 +1161,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Dinas Perumahan Rakyat, Kawasan Pemukiman dan Pertanahan</t>
+          <t>Dinas Perumahan Rakyat, Kawasan Pemukiman dan Pertanahanâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1189,7 +1189,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Dinas Sosial</t>
+          <t>Dinas Sosialâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1217,7 +1217,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Dinas Tenaga Kerja dan Transmigrasi</t>
+          <t>Dinas Tenaga Kerja dan Transmigrasiâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1245,7 +1245,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Inspektorat Daerah</t>
+          <t>Inspektorat Daerahâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1273,7 +1273,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Instalasi Farmasi</t>
+          <t>Instalasi Farmasiâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1301,7 +1301,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Kecamatan Arut Selatan</t>
+          <t>Kecamatan Arut Selatanâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1329,7 +1329,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Kecamatan Arut Utara</t>
+          <t>Kecamatan Arut Utaraâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1357,7 +1357,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Kecamatan Kotawaringin Lama</t>
+          <t>Kecamatan Kotawaringin Lamaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1385,7 +1385,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Kecamatan Kumai</t>
+          <t>Kecamatan Kumaiâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1413,7 +1413,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Kecamatan Pangkalan Banteng</t>
+          <t>Kecamatan Pangkalan Bantengâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1441,7 +1441,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Kecamatan Pangkalan Lada</t>
+          <t>Kecamatan Pangkalan Ladaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1469,7 +1469,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Kelurahan Baru</t>
+          <t>Kelurahan Baruâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1497,7 +1497,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Kelurahan Candi</t>
+          <t>Kelurahan Candiâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1525,7 +1525,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Kelurahan Kotawaringin Hilir</t>
+          <t>Kelurahan Kotawaringin Hilirâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1553,7 +1553,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Kelurahan Kotawaringin Hulu</t>
+          <t>Kelurahan Kotawaringin Huluâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1581,7 +1581,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Kelurahan Kumai Hilir</t>
+          <t>Kelurahan Kumai Hilirâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1609,7 +1609,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Kelurahan Kumai Hulu</t>
+          <t>Kelurahan Kumai Huluâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1637,7 +1637,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Kelurahan Madurejo</t>
+          <t>Kelurahan Madurejoâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1665,7 +1665,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Kelurahan Mendawai</t>
+          <t>Kelurahan Mendawai Seberangâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1693,7 +1693,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Kelurahan Mendawai Seberang</t>
+          <t>Kelurahan Mendawaiâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1721,7 +1721,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Kelurahan Pangkut</t>
+          <t>Kelurahan Pangkutâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1749,7 +1749,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Kelurahan Raja</t>
+          <t>Kelurahan Raja Seberangâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1777,7 +1777,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Kelurahan Raja Seberang</t>
+          <t>Kelurahan Rajaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1805,7 +1805,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Kelurahan Sidorejo</t>
+          <t>Kelurahan Sidorejoâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1833,7 +1833,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Laboratorium Bahan Konstruksi</t>
+          <t>Laboratorium Bahan Konstruksiâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1861,7 +1861,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Laboratorium Kesehatan Daerah</t>
+          <t>Laboratorium Kesehatan Daerahâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1889,7 +1889,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Laboratorium Lingkungan</t>
+          <t>Laboratorium Lingkunganâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1917,7 +1917,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Pelabuhan Penyeberangan Kumai</t>
+          <t>Pelabuhan Penyeberangan Kumaiâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1945,7 +1945,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Pengembangan Pakan dan Ternak Unggul</t>
+          <t>Pengembangan Pakan dan Ternak Unggulâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1973,7 +1973,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Pengujian Kendaraan Bermotor</t>
+          <t>Pengujian Kendaraan Bermotorâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -2001,7 +2001,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Puskesmas Arut Selatan</t>
+          <t>Puskesmas Arut Selatanâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2029,7 +2029,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Puskesmas Arut Utara</t>
+          <t>Puskesmas Arut Utaraâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -2057,7 +2057,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Puskesmas Ipuh Bangun Jaya</t>
+          <t>Puskesmas Ipuh Bangun Jayaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -2085,7 +2085,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Puskesmas Karang Mulya</t>
+          <t>Puskesmas Karang Mulyaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -2113,7 +2113,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Puskesmas Kotawaringin Lama</t>
+          <t>Puskesmas Kotawaringin Lamaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -2141,7 +2141,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Puskesmas Kumai</t>
+          <t>Puskesmas Kumaiâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -2169,7 +2169,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Puskesmas Kumpai Batu Atas</t>
+          <t>Puskesmas Kumpai Batu Atasâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -2197,7 +2197,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Puskesmas Madurejo</t>
+          <t>Puskesmas Madurejoâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -2225,7 +2225,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Puskesmas Mendawai</t>
+          <t>Puskesmas Mendawaiâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -2253,7 +2253,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Puskesmas Natai Pelingkau</t>
+          <t>Puskesmas Natai Pelingkauâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -2281,7 +2281,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Puskesmas Pandu Sanjaya</t>
+          <t>Puskesmas Pandu Sanjayaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -2309,7 +2309,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Puskesmas Pangkalan Lada</t>
+          <t>Puskesmas Pangkalan Ladaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -2337,7 +2337,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Puskesmas Riam Durian</t>
+          <t>Puskesmas Riam Durianâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -2365,7 +2365,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Puskesmas Runtu</t>
+          <t>Puskesmas Runtuâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -2393,7 +2393,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Puskesmas Sambi</t>
+          <t>Puskesmas Sambiâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -2421,7 +2421,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Puskesmas Semanggang</t>
+          <t>Puskesmas Semanggangâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -2449,7 +2449,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Puskesmas Sungai Rangit</t>
+          <t>Puskesmas Sungai Rangitâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -2477,7 +2477,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Puskesmas Teluk Bogam</t>
+          <t>Puskesmas Teluk Bogamâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -2505,7 +2505,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Rumah Potong Hewan Ruminansia</t>
+          <t>Rumah Potong Hewan Ruminansiaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -2533,7 +2533,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Rumah Sakit Kutaringin</t>
+          <t>Rumah Sakit Kutaringinâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -2561,11 +2561,11 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Rumah Sakit Umum Daerah Sultan Imanuddin</t>
+          <t>Rumah Sakit Umum Daerah Sultan Imanuddinâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>139926000000</v>
+        <v>136086000000</v>
       </c>
       <c r="C77" t="n">
         <v>85676806400</v>
@@ -2589,7 +2589,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Satuan Polisi Pamong Praja</t>
+          <t>Satuan Polisi Pamong Prajaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -2617,7 +2617,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Sekretariat Daerah</t>
+          <t>Sekretariat Daerahâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -2645,11 +2645,11 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Sekretariat DPRD</t>
+          <t>Sekretariat DPRDâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>16938018018</v>
+        <v>16485728018</v>
       </c>
       <c r="C80" t="n">
         <v>8905641688</v>
@@ -2673,7 +2673,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Workshop dan Peralatan Konstruksi</t>
+          <t>Workshop dan Peralatan Konstruksiâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
         </is>
       </c>
       <c r="B81" t="n">

</xml_diff>

<commit_message>
auto update 21/04/2026 10.00.43,79
</commit_message>
<xml_diff>
--- a/output/Rekap RUP Tahun 2026 (2026-04-21) Legacy.xlsx
+++ b/output/Rekap RUP Tahun 2026 (2026-04-21) Legacy.xlsx
@@ -461,7 +461,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Badan Kepegawaian dan Pengembangan Sumber Daya Manusiaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Badan Kepegawaian dan Pengembangan Sumber Daya Manusiaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -489,7 +489,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Badan Kesatuan Bangsa dan Politikâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Badan Kesatuan Bangsa dan Politikâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -517,7 +517,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Badan Keuangan dan Aset Daerahâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Badan Keuangan dan Aset Daerahâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -545,7 +545,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Badan Penanggulangan Bencana Daerahâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Badan Penanggulangan Bencana Daerahâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -573,7 +573,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Badan Pendapatan Daerahâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Badan Pendapatan Daerahâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -601,7 +601,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Badan Perencanaan Pembangunan, Riset dan Inovasi Daerahâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Badan Perencanaan Pembangunan, Riset dan Inovasi Daerahâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -629,7 +629,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Balai Latihan Kerjaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Balai Latihan Kerjaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -657,7 +657,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Dermaga Indera Sariâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Dermaga Indera Sariâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -685,7 +685,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Dinas Kepemudaan dan Olahragaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Dinas Kepemudaan dan Olahragaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -713,7 +713,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Dinas Kependudukan dan Pencatatan Sipilâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Dinas Kependudukan dan Pencatatan Sipilâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -741,7 +741,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Dinas Kesehatanâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Dinas Kesehatanâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -769,7 +769,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Dinas Komunikasi, Informatika, Statistik dan Persandianâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Dinas Komunikasi, Informatika, Statistik dan Persandianâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -797,7 +797,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Dinas Lingkungan Hidupâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Dinas Lingkungan Hidupâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -825,7 +825,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Dinas Pariwisataâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Dinas Pariwisataâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -853,7 +853,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Dinas Pekerjaan Umum dan Penataan Ruangâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Dinas Pekerjaan Umum dan Penataan Ruangâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -881,7 +881,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Dinas Pemadam Kebakaran dan Penyelamatanâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Dinas Pemadam Kebakaran dan Penyelamatanâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -909,7 +909,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Dinas Pemberdayaan Masyarakat dan Desaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Dinas Pemberdayaan Masyarakat dan Desaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -937,7 +937,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Dinas Pemberdayaan Perempuan dan Perlindungan Anak, Pengendalian Penduduk dan Keluarga Berencanaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Dinas Pemberdayaan Perempuan dan Perlindungan Anak, Pengendalian Penduduk dan Keluarga Berencanaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -965,7 +965,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Dinas Penanaman Modal dan Pelayanan Terpadu Satu Pintuâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Dinas Penanaman Modal dan Pelayanan Terpadu Satu Pintuâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -993,7 +993,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Dinas Pendidikan dan Kebudayaanâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Dinas Pendidikan dan Kebudayaanâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1021,7 +1021,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Dinas Perhubunganâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Dinas Perhubunganâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1049,7 +1049,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Dinas Perikanan dan Ketahanan Panganâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Dinas Perikanan dan Ketahanan Panganâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1077,7 +1077,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Dinas Perindustrian, Perdagangan, Koperasi, Usaha Kecil dan Menengahâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Dinas Perindustrian, Perdagangan, Koperasi, Usaha Kecil dan Menengahâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1105,7 +1105,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Dinas Perpustakaan dan Kearsipanâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Dinas Perpustakaan dan Kearsipanâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1133,7 +1133,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Dinas Pertanianâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Dinas Pertanianâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1161,7 +1161,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Dinas Perumahan Rakyat, Kawasan Pemukiman dan Pertanahanâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Dinas Perumahan Rakyat, Kawasan Pemukiman dan Pertanahanâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1189,7 +1189,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Dinas Sosialâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Dinas Sosialâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1217,7 +1217,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Dinas Tenaga Kerja dan Transmigrasiâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Dinas Tenaga Kerja dan Transmigrasiâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1245,7 +1245,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Inspektorat Daerahâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Inspektorat Daerahâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1273,7 +1273,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Instalasi Farmasiâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Instalasi Farmasiâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1301,7 +1301,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Kecamatan Arut Selatanâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Kecamatan Arut Selatanâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1329,7 +1329,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Kecamatan Arut Utaraâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Kecamatan Arut Utaraâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1357,7 +1357,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Kecamatan Kotawaringin Lamaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Kecamatan Kotawaringin Lamaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1385,7 +1385,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Kecamatan Kumaiâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Kecamatan Kumaiâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1413,7 +1413,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Kecamatan Pangkalan Bantengâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Kecamatan Pangkalan Bantengâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1441,7 +1441,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Kecamatan Pangkalan Ladaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Kecamatan Pangkalan Ladaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1469,7 +1469,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Kelurahan Baruâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Kelurahan Baruâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1497,7 +1497,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Kelurahan Candiâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Kelurahan Candiâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1525,7 +1525,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Kelurahan Kotawaringin Hilirâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Kelurahan Kotawaringin Hilirâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1553,7 +1553,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Kelurahan Kotawaringin Huluâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Kelurahan Kotawaringin Huluâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1581,7 +1581,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Kelurahan Kumai Hilirâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Kelurahan Kumai Hilirâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1609,7 +1609,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Kelurahan Kumai Huluâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Kelurahan Kumai Huluâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1637,7 +1637,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Kelurahan Madurejoâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Kelurahan Madurejoâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1665,7 +1665,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Kelurahan Mendawai Seberangâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Kelurahan Mendawai Seberangâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1693,7 +1693,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Kelurahan Mendawaiâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Kelurahan Mendawaiâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1721,7 +1721,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Kelurahan Pangkutâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Kelurahan Pangkutâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1749,7 +1749,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Kelurahan Raja Seberangâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Kelurahan Raja Seberangâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1777,7 +1777,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Kelurahan Rajaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Kelurahan Rajaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1805,7 +1805,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Kelurahan Sidorejoâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Kelurahan Sidorejoâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1833,7 +1833,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Laboratorium Bahan Konstruksiâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Laboratorium Bahan Konstruksiâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1861,7 +1861,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Laboratorium Kesehatan Daerahâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Laboratorium Kesehatan Daerahâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1889,7 +1889,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Laboratorium Lingkunganâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Laboratorium Lingkunganâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1917,7 +1917,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Pelabuhan Penyeberangan Kumaiâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Pelabuhan Penyeberangan Kumaiâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1945,7 +1945,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Pengembangan Pakan dan Ternak Unggulâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Pengembangan Pakan dan Ternak Unggulâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1973,7 +1973,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Pengujian Kendaraan Bermotorâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Pengujian Kendaraan Bermotorâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -2001,7 +2001,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Puskesmas Arut Selatanâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Puskesmas Arut Selatanâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2029,7 +2029,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Puskesmas Arut Utaraâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Puskesmas Arut Utaraâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -2057,7 +2057,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Puskesmas Ipuh Bangun Jayaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Puskesmas Ipuh Bangun Jayaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -2085,7 +2085,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Puskesmas Karang Mulyaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Puskesmas Karang Mulyaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -2113,7 +2113,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Puskesmas Kotawaringin Lamaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Puskesmas Kotawaringin Lamaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -2141,7 +2141,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Puskesmas Kumaiâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Puskesmas Kumaiâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -2169,7 +2169,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Puskesmas Kumpai Batu Atasâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Puskesmas Kumpai Batu Atasâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -2197,7 +2197,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Puskesmas Madurejoâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Puskesmas Madurejoâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -2225,7 +2225,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Puskesmas Mendawaiâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Puskesmas Mendawaiâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -2253,7 +2253,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Puskesmas Natai Pelingkauâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Puskesmas Natai Pelingkauâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -2281,7 +2281,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Puskesmas Pandu Sanjayaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Puskesmas Pandu Sanjayaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -2309,7 +2309,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Puskesmas Pangkalan Ladaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Puskesmas Pangkalan Ladaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -2337,7 +2337,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Puskesmas Riam Durianâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Puskesmas Riam Durianâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -2365,7 +2365,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Puskesmas Runtuâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Puskesmas Runtuâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -2393,7 +2393,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Puskesmas Sambiâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Puskesmas Sambiâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -2421,7 +2421,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Puskesmas Semanggangâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Puskesmas Semanggangâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -2449,7 +2449,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Puskesmas Sungai Rangitâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Puskesmas Sungai Rangitâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -2477,7 +2477,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Puskesmas Teluk Bogamâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Puskesmas Teluk Bogamâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -2505,7 +2505,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Rumah Potong Hewan Ruminansiaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Rumah Potong Hewan Ruminansiaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -2533,7 +2533,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Rumah Sakit Kutaringinâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Rumah Sakit Kutaringinâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -2561,7 +2561,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Rumah Sakit Umum Daerah Sultan Imanuddinâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Rumah Sakit Umum Daerah Sultan Imanuddinâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -2589,7 +2589,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Satuan Polisi Pamong Prajaâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Satuan Polisi Pamong Prajaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -2617,7 +2617,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Sekretariat Daerahâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Sekretariat Daerahâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -2645,7 +2645,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Sekretariat DPRDâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Sekretariat DPRDâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -2673,7 +2673,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Workshop dan Peralatan Konstruksiâ£âââââââââââ â âââââââââ â â âââ âââââ âââ ââ âââ ââââ âââââ â ââââ ââââââââââââââââ¤</t>
+          <t>Workshop dan Peralatan Konstruksiâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
         </is>
       </c>
       <c r="B81" t="n">

</xml_diff>

<commit_message>
auto update 21/04/2026 11.00.22,52
</commit_message>
<xml_diff>
--- a/output/Rekap RUP Tahun 2026 (2026-04-21) Legacy.xlsx
+++ b/output/Rekap RUP Tahun 2026 (2026-04-21) Legacy.xlsx
@@ -461,7 +461,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Badan Kepegawaian dan Pengembangan Sumber Daya Manusiaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Badan Kepegawaian dan Pengembangan Sumber Daya Manusiaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -489,7 +489,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Badan Kesatuan Bangsa dan Politikâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Badan Kesatuan Bangsa dan Politikâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -517,7 +517,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Badan Keuangan dan Aset Daerahâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Badan Keuangan dan Aset Daerahâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -545,7 +545,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Badan Penanggulangan Bencana Daerahâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Badan Penanggulangan Bencana Daerahâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -573,7 +573,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Badan Pendapatan Daerahâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Badan Pendapatan Daerahâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -601,7 +601,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Badan Perencanaan Pembangunan, Riset dan Inovasi Daerahâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Badan Perencanaan Pembangunan, Riset dan Inovasi Daerahâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -629,7 +629,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Balai Latihan Kerjaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Balai Latihan Kerjaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -657,7 +657,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Dermaga Indera Sariâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Dermaga Indera Sariâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -685,7 +685,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Dinas Kepemudaan dan Olahragaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Dinas Kepemudaan dan Olahragaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -713,7 +713,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Dinas Kependudukan dan Pencatatan Sipilâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Dinas Kependudukan dan Pencatatan Sipilâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -741,7 +741,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Dinas Kesehatanâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Dinas Kesehatanâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -769,11 +769,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Dinas Komunikasi, Informatika, Statistik dan Persandianâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Dinas Komunikasi, Informatika, Statistik dan Persandianâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>4809371581</v>
+        <v>7585371581</v>
       </c>
       <c r="C13" t="n">
         <v>4363300381</v>
@@ -797,7 +797,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Dinas Lingkungan Hidupâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Dinas Lingkungan Hidupâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -825,7 +825,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Dinas Pariwisataâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Dinas Pariwisataâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -853,11 +853,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Dinas Pekerjaan Umum dan Penataan Ruangâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Dinas Pekerjaan Umum dan Penataan Ruangâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>105714344580</v>
+        <v>106337273694</v>
       </c>
       <c r="C16" t="n">
         <v>105032048100</v>
@@ -881,7 +881,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Dinas Pemadam Kebakaran dan Penyelamatanâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Dinas Pemadam Kebakaran dan Penyelamatanâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -909,7 +909,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Dinas Pemberdayaan Masyarakat dan Desaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Dinas Pemberdayaan Masyarakat dan Desaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -937,7 +937,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Dinas Pemberdayaan Perempuan dan Perlindungan Anak, Pengendalian Penduduk dan Keluarga Berencanaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Dinas Pemberdayaan Perempuan dan Perlindungan Anak, Pengendalian Penduduk dan Keluarga Berencanaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -965,7 +965,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Dinas Penanaman Modal dan Pelayanan Terpadu Satu Pintuâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Dinas Penanaman Modal dan Pelayanan Terpadu Satu Pintuâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -993,7 +993,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Dinas Pendidikan dan Kebudayaanâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Dinas Pendidikan dan Kebudayaanâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1021,7 +1021,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Dinas Perhubunganâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Dinas Perhubunganâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1049,7 +1049,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Dinas Perikanan dan Ketahanan Panganâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Dinas Perikanan dan Ketahanan Panganâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1077,7 +1077,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Dinas Perindustrian, Perdagangan, Koperasi, Usaha Kecil dan Menengahâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Dinas Perindustrian, Perdagangan, Koperasi, Usaha Kecil dan Menengahâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1105,7 +1105,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Dinas Perpustakaan dan Kearsipanâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Dinas Perpustakaan dan Kearsipanâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1133,7 +1133,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Dinas Pertanianâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Dinas Pertanianâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1161,7 +1161,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Dinas Perumahan Rakyat, Kawasan Pemukiman dan Pertanahanâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Dinas Perumahan Rakyat, Kawasan Pemukiman dan Pertanahanâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1189,7 +1189,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Dinas Sosialâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Dinas Sosialâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1217,7 +1217,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Dinas Tenaga Kerja dan Transmigrasiâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Dinas Tenaga Kerja dan Transmigrasiâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1245,7 +1245,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Inspektorat Daerahâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Inspektorat Daerahâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1273,7 +1273,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Instalasi Farmasiâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Instalasi Farmasiâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1301,7 +1301,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Kecamatan Arut Selatanâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Kecamatan Arut Selatanâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1329,7 +1329,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Kecamatan Arut Utaraâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Kecamatan Arut Utaraâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1357,7 +1357,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Kecamatan Kotawaringin Lamaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Kecamatan Kotawaringin Lamaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1385,7 +1385,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Kecamatan Kumaiâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Kecamatan Kumaiâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1413,7 +1413,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Kecamatan Pangkalan Bantengâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Kecamatan Pangkalan Bantengâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1441,7 +1441,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Kecamatan Pangkalan Ladaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Kecamatan Pangkalan Ladaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1469,7 +1469,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Kelurahan Baruâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Kelurahan Baruâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1497,7 +1497,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Kelurahan Candiâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Kelurahan Candiâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1525,7 +1525,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Kelurahan Kotawaringin Hilirâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Kelurahan Kotawaringin Hilirâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1553,7 +1553,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Kelurahan Kotawaringin Huluâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Kelurahan Kotawaringin Huluâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1581,7 +1581,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Kelurahan Kumai Hilirâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Kelurahan Kumai Hilirâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1609,7 +1609,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Kelurahan Kumai Huluâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Kelurahan Kumai Huluâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1637,7 +1637,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Kelurahan Madurejoâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Kelurahan Madurejoâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1665,7 +1665,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Kelurahan Mendawai Seberangâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Kelurahan Mendawai Seberangâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1693,7 +1693,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Kelurahan Mendawaiâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Kelurahan Mendawaiâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1721,7 +1721,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Kelurahan Pangkutâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Kelurahan Pangkutâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1749,7 +1749,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Kelurahan Raja Seberangâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Kelurahan Raja Seberangâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1777,7 +1777,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Kelurahan Rajaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Kelurahan Rajaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1805,7 +1805,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Kelurahan Sidorejoâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Kelurahan Sidorejoâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1833,7 +1833,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Laboratorium Bahan Konstruksiâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Laboratorium Bahan Konstruksiâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1861,7 +1861,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Laboratorium Kesehatan Daerahâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Laboratorium Kesehatan Daerahâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1889,7 +1889,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Laboratorium Lingkunganâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Laboratorium Lingkunganâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1917,7 +1917,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Pelabuhan Penyeberangan Kumaiâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Pelabuhan Penyeberangan Kumaiâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1945,7 +1945,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Pengembangan Pakan dan Ternak Unggulâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Pengembangan Pakan dan Ternak Unggulâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1973,7 +1973,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Pengujian Kendaraan Bermotorâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Pengujian Kendaraan Bermotorâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -2001,7 +2001,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Puskesmas Arut Selatanâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Puskesmas Arut Selatanâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2029,7 +2029,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Puskesmas Arut Utaraâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Puskesmas Arut Utaraâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -2057,7 +2057,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Puskesmas Ipuh Bangun Jayaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Puskesmas Ipuh Bangun Jayaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -2085,7 +2085,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Puskesmas Karang Mulyaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Puskesmas Karang Mulyaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -2113,7 +2113,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Puskesmas Kotawaringin Lamaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Puskesmas Kotawaringin Lamaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -2141,7 +2141,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Puskesmas Kumaiâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Puskesmas Kumaiâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -2169,7 +2169,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Puskesmas Kumpai Batu Atasâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Puskesmas Kumpai Batu Atasâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -2197,7 +2197,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Puskesmas Madurejoâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Puskesmas Madurejoâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -2225,7 +2225,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Puskesmas Mendawaiâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Puskesmas Mendawaiâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -2253,7 +2253,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Puskesmas Natai Pelingkauâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Puskesmas Natai Pelingkauâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -2281,7 +2281,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Puskesmas Pandu Sanjayaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Puskesmas Pandu Sanjayaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -2309,7 +2309,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Puskesmas Pangkalan Ladaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Puskesmas Pangkalan Ladaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -2337,7 +2337,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Puskesmas Riam Durianâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Puskesmas Riam Durianâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -2365,7 +2365,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Puskesmas Runtuâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Puskesmas Runtuâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -2393,7 +2393,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Puskesmas Sambiâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Puskesmas Sambiâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -2421,7 +2421,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Puskesmas Semanggangâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Puskesmas Semanggangâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -2449,7 +2449,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Puskesmas Sungai Rangitâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Puskesmas Sungai Rangitâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -2477,7 +2477,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Puskesmas Teluk Bogamâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Puskesmas Teluk Bogamâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -2505,7 +2505,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Rumah Potong Hewan Ruminansiaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Rumah Potong Hewan Ruminansiaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -2533,7 +2533,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Rumah Sakit Kutaringinâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Rumah Sakit Kutaringinâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -2561,11 +2561,11 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Rumah Sakit Umum Daerah Sultan Imanuddinâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Rumah Sakit Umum Daerah Sultan Imanuddinâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>136086000000</v>
+        <v>139926000000</v>
       </c>
       <c r="C77" t="n">
         <v>85676806400</v>
@@ -2589,7 +2589,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Satuan Polisi Pamong Prajaâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Satuan Polisi Pamong Prajaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -2617,7 +2617,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Sekretariat Daerahâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Sekretariat Daerahâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -2645,11 +2645,11 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Sekretariat DPRDâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Sekretariat DPRDâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>16485728018</v>
+        <v>16938018018</v>
       </c>
       <c r="C80" t="n">
         <v>8905641688</v>
@@ -2673,7 +2673,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Workshop dan Peralatan Konstruksiâ£âââââââââ ââ â â â âââââ âââââ ââââââââ â âââââââââ ââ ââââââââ â ââ âââââ ââââ âââââ¤</t>
+          <t>Workshop dan Peralatan Konstruksiâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
         </is>
       </c>
       <c r="B81" t="n">

</xml_diff>

<commit_message>
auto update 21/04/2026 12.00.24,43
</commit_message>
<xml_diff>
--- a/output/Rekap RUP Tahun 2026 (2026-04-21) Legacy.xlsx
+++ b/output/Rekap RUP Tahun 2026 (2026-04-21) Legacy.xlsx
@@ -461,7 +461,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Badan Kepegawaian dan Pengembangan Sumber Daya Manusiaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Badan Kepegawaian dan Pengembangan Sumber Daya Manusiaâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -489,7 +489,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Badan Kesatuan Bangsa dan Politikâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Badan Kesatuan Bangsa dan Politikâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -517,7 +517,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Badan Keuangan dan Aset Daerahâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Badan Keuangan dan Aset Daerahâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -545,7 +545,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Badan Penanggulangan Bencana Daerahâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Badan Penanggulangan Bencana Daerahâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -573,7 +573,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Badan Pendapatan Daerahâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Badan Pendapatan Daerahâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -601,7 +601,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Badan Perencanaan Pembangunan, Riset dan Inovasi Daerahâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Badan Perencanaan Pembangunan, Riset dan Inovasi Daerahâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -629,7 +629,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Balai Latihan Kerjaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Balai Latihan Kerjaâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -657,7 +657,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Dermaga Indera Sariâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Dermaga Indera Sariâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -685,7 +685,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Dinas Kepemudaan dan Olahragaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Dinas Kepemudaan dan Olahragaâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -713,7 +713,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Dinas Kependudukan dan Pencatatan Sipilâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Dinas Kependudukan dan Pencatatan Sipilâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -741,7 +741,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Dinas Kesehatanâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Dinas Kesehatanâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -769,7 +769,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Dinas Komunikasi, Informatika, Statistik dan Persandianâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Dinas Komunikasi, Informatika, Statistik dan Persandianâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -797,7 +797,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Dinas Lingkungan Hidupâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Dinas Lingkungan Hidupâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -825,7 +825,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Dinas Pariwisataâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Dinas Pariwisataâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -853,7 +853,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Dinas Pekerjaan Umum dan Penataan Ruangâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Dinas Pekerjaan Umum dan Penataan Ruangâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -881,7 +881,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Dinas Pemadam Kebakaran dan Penyelamatanâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Dinas Pemadam Kebakaran dan Penyelamatanâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -909,7 +909,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Dinas Pemberdayaan Masyarakat dan Desaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Dinas Pemberdayaan Masyarakat dan Desaâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -937,7 +937,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Dinas Pemberdayaan Perempuan dan Perlindungan Anak, Pengendalian Penduduk dan Keluarga Berencanaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Dinas Pemberdayaan Perempuan dan Perlindungan Anak, Pengendalian Penduduk dan Keluarga Berencanaâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -965,7 +965,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Dinas Penanaman Modal dan Pelayanan Terpadu Satu Pintuâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Dinas Penanaman Modal dan Pelayanan Terpadu Satu Pintuâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -993,7 +993,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Dinas Pendidikan dan Kebudayaanâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Dinas Pendidikan dan Kebudayaanâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1021,7 +1021,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Dinas Perhubunganâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Dinas Perhubunganâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1049,7 +1049,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Dinas Perikanan dan Ketahanan Panganâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Dinas Perikanan dan Ketahanan Panganâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1077,7 +1077,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Dinas Perindustrian, Perdagangan, Koperasi, Usaha Kecil dan Menengahâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Dinas Perindustrian, Perdagangan, Koperasi, Usaha Kecil dan Menengahâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1105,7 +1105,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Dinas Perpustakaan dan Kearsipanâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Dinas Perpustakaan dan Kearsipanâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1133,7 +1133,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Dinas Pertanianâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Dinas Pertanianâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1161,7 +1161,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Dinas Perumahan Rakyat, Kawasan Pemukiman dan Pertanahanâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Dinas Perumahan Rakyat, Kawasan Pemukiman dan Pertanahanâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1189,7 +1189,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Dinas Sosialâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Dinas Sosialâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1217,7 +1217,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Dinas Tenaga Kerja dan Transmigrasiâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Dinas Tenaga Kerja dan Transmigrasiâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1245,7 +1245,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Inspektorat Daerahâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Inspektorat Daerahâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1273,7 +1273,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Instalasi Farmasiâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Instalasi Farmasiâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1301,7 +1301,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Kecamatan Arut Selatanâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Kecamatan Arut Selatanâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1329,7 +1329,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Kecamatan Arut Utaraâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Kecamatan Arut Utaraâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1357,7 +1357,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Kecamatan Kotawaringin Lamaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Kecamatan Kotawaringin Lamaâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1385,7 +1385,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Kecamatan Kumaiâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Kecamatan Kumaiâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1413,7 +1413,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Kecamatan Pangkalan Bantengâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Kecamatan Pangkalan Bantengâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1441,7 +1441,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Kecamatan Pangkalan Ladaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Kecamatan Pangkalan Ladaâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1469,7 +1469,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Kelurahan Baruâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Kelurahan Baruâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1497,7 +1497,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Kelurahan Candiâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Kelurahan Candiâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1525,7 +1525,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Kelurahan Kotawaringin Hilirâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Kelurahan Kotawaringin Hilirâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1553,7 +1553,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Kelurahan Kotawaringin Huluâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Kelurahan Kotawaringin Huluâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1581,7 +1581,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Kelurahan Kumai Hilirâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Kelurahan Kumai Hilirâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1609,7 +1609,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Kelurahan Kumai Huluâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Kelurahan Kumai Huluâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1637,7 +1637,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Kelurahan Madurejoâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Kelurahan Madurejoâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1665,7 +1665,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Kelurahan Mendawai Seberangâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Kelurahan Mendawai Seberangâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1693,7 +1693,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Kelurahan Mendawaiâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Kelurahan Mendawaiâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1721,7 +1721,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Kelurahan Pangkutâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Kelurahan Pangkutâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1749,7 +1749,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Kelurahan Raja Seberangâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Kelurahan Raja Seberangâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1777,7 +1777,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Kelurahan Rajaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Kelurahan Rajaâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1805,7 +1805,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Kelurahan Sidorejoâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Kelurahan Sidorejoâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1833,7 +1833,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Laboratorium Bahan Konstruksiâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Laboratorium Bahan Konstruksiâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1861,7 +1861,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Laboratorium Kesehatan Daerahâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Laboratorium Kesehatan Daerahâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1889,7 +1889,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Laboratorium Lingkunganâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Laboratorium Lingkunganâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1917,7 +1917,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Pelabuhan Penyeberangan Kumaiâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Pelabuhan Penyeberangan Kumaiâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1945,7 +1945,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Pengembangan Pakan dan Ternak Unggulâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Pengembangan Pakan dan Ternak Unggulâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1973,7 +1973,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Pengujian Kendaraan Bermotorâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Pengujian Kendaraan Bermotorâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -2001,7 +2001,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Puskesmas Arut Selatanâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Puskesmas Arut Selatanâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2029,7 +2029,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Puskesmas Arut Utaraâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Puskesmas Arut Utaraâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -2057,7 +2057,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Puskesmas Ipuh Bangun Jayaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Puskesmas Ipuh Bangun Jayaâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -2085,7 +2085,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Puskesmas Karang Mulyaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Puskesmas Karang Mulyaâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -2113,7 +2113,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Puskesmas Kotawaringin Lamaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Puskesmas Kotawaringin Lamaâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -2141,7 +2141,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Puskesmas Kumaiâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Puskesmas Kumaiâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -2169,7 +2169,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Puskesmas Kumpai Batu Atasâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Puskesmas Kumpai Batu Atasâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -2197,7 +2197,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Puskesmas Madurejoâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Puskesmas Madurejoâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -2225,7 +2225,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Puskesmas Mendawaiâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Puskesmas Mendawaiâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -2253,7 +2253,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Puskesmas Natai Pelingkauâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Puskesmas Natai Pelingkauâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -2281,7 +2281,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Puskesmas Pandu Sanjayaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Puskesmas Pandu Sanjayaâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -2309,7 +2309,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Puskesmas Pangkalan Ladaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Puskesmas Pangkalan Ladaâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -2337,7 +2337,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Puskesmas Riam Durianâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Puskesmas Riam Durianâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -2365,7 +2365,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Puskesmas Runtuâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Puskesmas Runtuâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -2393,7 +2393,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Puskesmas Sambiâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Puskesmas Sambiâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -2421,7 +2421,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Puskesmas Semanggangâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Puskesmas Semanggangâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -2449,7 +2449,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Puskesmas Sungai Rangitâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Puskesmas Sungai Rangitâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -2477,7 +2477,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Puskesmas Teluk Bogamâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Puskesmas Teluk Bogamâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -2505,7 +2505,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Rumah Potong Hewan Ruminansiaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Rumah Potong Hewan Ruminansiaâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -2533,7 +2533,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Rumah Sakit Kutaringinâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Rumah Sakit Kutaringinâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -2561,7 +2561,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Rumah Sakit Umum Daerah Sultan Imanuddinâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Rumah Sakit Umum Daerah Sultan Imanuddinâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -2589,7 +2589,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Satuan Polisi Pamong Prajaâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Satuan Polisi Pamong Prajaâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -2617,7 +2617,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Sekretariat Daerahâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Sekretariat Daerahâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -2645,7 +2645,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Sekretariat DPRDâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Sekretariat DPRDâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -2673,7 +2673,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Workshop dan Peralatan Konstruksiâ£âââââ â âââ âââ âââââââ ââââ âââ ââ âââ âââ âââââââ âââââ âââ âââââââââââââââ âââââ¤</t>
+          <t>Workshop dan Peralatan Konstruksiâ£âââââââ âââ â ââââââââââââ â â âââ âââââ âââ âââââââ â ââââââ â â â ââââ â â â ââââââ ââ â¤</t>
         </is>
       </c>
       <c r="B81" t="n">

</xml_diff>